<commit_message>
Track landing-page redesign and update readiness sheets
</commit_message>
<xml_diff>
--- a/docs/executive.xlsx
+++ b/docs/executive.xlsx
@@ -1041,12 +1041,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Tune Civis AI quality for live users</t>
+          <t>Redesign landing page and premium positioning</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Product + Engineering</t>
+          <t>Product + Design + Engineering</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1056,44 +1056,44 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Ongoing</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Stable AI provider configuration</t>
+          <t>Core platform credibility first</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>AI is materially improved but still needs polish</t>
+          <t>The current landing page does not yet match the quality of the product ambition</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Collect real prompts and refine responses</t>
+          <t>Treat it as a dedicated brand/conversion redesign later</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Execute NDPA/VAPT hardening backlog</t>
+          <t>Tune Civis AI quality for live users</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Engineering + Security</t>
+          <t>Product + Engineering</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1103,12 +1103,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1118,62 +1118,109 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Security docs already created</t>
+          <t>Stable AI provider configuration</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Architecture and API docs exist; implementation backlog remains</t>
+          <t>AI is materially improved but still needs polish</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Prioritize access control, monitoring, and incident readiness</t>
+          <t>Collect real prompts and refine responses</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Execute NDPA/VAPT hardening backlog</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Engineering + Security</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Security docs already created</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Architecture and API docs exist; implementation backlog remains</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Prioritize access control, monitoring, and incident readiness</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>Keep documentation and OpenAPI in sync</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>2026-05-30</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Feature shipping discipline</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>Docs exist and should now be maintained with each batch</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>Make docs updates part of release definition</t>
         </is>

</xml_diff>